<commit_message>
Rename glycerol stock columns to Rack_Shelf and Position on Drawer
The lab's own sheets use these names. Only the labels change: the stored
fields (shelf, shelfPlace) stay the same, so existing stocks keep their
values. The old header names still map on bulk upload. Template
regenerated; asset versions bumped to v=13.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/elias-lab-inventory-template.xlsx
+++ b/assets/elias-lab-inventory-template.xlsx
@@ -721,13 +721,13 @@
         <v>Glycerol Stocks</v>
       </c>
       <c r="B30" t="str">
-        <v>Shelf</v>
+        <v>Rack_Shelf</v>
       </c>
       <c r="C30" t="str">
         <v/>
       </c>
       <c r="D30" t="str">
-        <v>2</v>
+        <v>R2_S3</v>
       </c>
     </row>
     <row r="31">
@@ -735,7 +735,7 @@
         <v>Glycerol Stocks</v>
       </c>
       <c r="B31" t="str">
-        <v>Place on Shelf</v>
+        <v>Position on Drawer</v>
       </c>
       <c r="C31" t="str">
         <v/>
@@ -1092,7 +1092,7 @@
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="19.83203125" customWidth="1"/>
     <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
     <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="16.83203125" customWidth="1"/>
@@ -1120,10 +1120,10 @@
         <v>Freezer (-80°C)</v>
       </c>
       <c r="G1" t="str">
-        <v>Shelf</v>
+        <v>Rack_Shelf</v>
       </c>
       <c r="H1" t="str">
-        <v>Place on Shelf</v>
+        <v>Position on Drawer</v>
       </c>
       <c r="I1" t="str">
         <v>Box</v>

</xml_diff>